<commit_message>
Atualização dos painéis em 21/10/2026 10:56 por Ruy Silveira Neto
</commit_message>
<xml_diff>
--- a/dados/mp1376.xlsx
+++ b/dados/mp1376.xlsx
@@ -466,7 +466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Operações de crédito rural contratadas para quitar ou amortizar dívidas de produtores atingidos por eventos climáticos e queda de preços (Res. CMN 5.330/2026).</t>
+          <t>Operações de crédito rural contratadas para quitar ou amortizar dívidas de produtores atingidos por eventos climáticos e queda de preços (Res. CMN 5.330/2026). Não inclui as renegociações de Cédulas de Produto Rural (CPR, art. 6º da MP), que não são registradas no SICOR.</t>
         </is>
       </c>
     </row>
@@ -476,14 +476,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fonte: Banco Central do Brasil, SICOR (microdados de renegociação, bases legais 050 e 051). Elaboração: Sistema FARSUL.</t>
+          <t>Fonte: Banco Central do Brasil, SICOR (microdados de renegociação, bases legais 050 e 051; não inclui CPR). Elaboração: Sistema FARSUL.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dados até 30/09/2026. Arquivo gerado em 20/10/2026. O Banco Central publica os microdados uma vez por mês e revisa os meses anteriores.</t>
+          <t>Dados até 30/09/2026. Arquivo gerado em 21/10/2026. O Banco Central publica os microdados uma vez por mês e revisa os meses anteriores.</t>
         </is>
       </c>
     </row>
@@ -11162,13 +11162,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D6B04E8-D059-4546-95A4-AC8C051C1BA9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6484F4C4-D5ED-46BB-B6CB-EF82CC799E21}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0DCAA875-6D34-4BDE-9514-2C717039E5DD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86F7BC9C-75C8-481F-8CC2-85549B785F32}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7B665FE4-B7F5-45E4-A9FD-537FB56A8062}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2525F93-5B62-4764-9F8F-EA288051146A}"/>
 </file>
</xml_diff>

<commit_message>
Atualização dos painéis em 27/10/2026 10:09 por Ruy Silveira Neto
</commit_message>
<xml_diff>
--- a/dados/mp1376.xlsx
+++ b/dados/mp1376.xlsx
@@ -483,7 +483,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dados até 30/09/2026. Arquivo gerado em 21/10/2026. O Banco Central publica os microdados uma vez por mês e revisa os meses anteriores.</t>
+          <t>Dados até 30/09/2026. Arquivo gerado em 27/10/2026. O Banco Central publica os microdados uma vez por mês e revisa os meses anteriores.</t>
         </is>
       </c>
     </row>
@@ -606,10 +606,10 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>3922730307.699988</v>
+        <v>3908272549.929989</v>
       </c>
       <c r="C2" s="8" t="n">
-        <v>0.7055104122356775</v>
+        <v>0.7053053937090903</v>
       </c>
     </row>
     <row r="3">
@@ -619,10 +619,10 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>1465640528.77</v>
+        <v>1461337927.17</v>
       </c>
       <c r="C3" s="8" t="n">
-        <v>0.2635982013884911</v>
+        <v>0.2637199706256735</v>
       </c>
     </row>
     <row r="4">
@@ -632,10 +632,10 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>64000433.88999994</v>
+        <v>63878436.72999994</v>
       </c>
       <c r="C4" s="8" t="n">
-        <v>0.01151059821990938</v>
+        <v>0.01152780554370009</v>
       </c>
     </row>
     <row r="5">
@@ -648,7 +648,7 @@
         <v>61861737.91999999</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.01112594973350193</v>
+        <v>0.0111638625151605</v>
       </c>
     </row>
     <row r="6">
@@ -661,7 +661,7 @@
         <v>37399267.38000001</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>0.006726328469429438</v>
+        <v>0.00674924910350865</v>
       </c>
     </row>
     <row r="7">
@@ -671,10 +671,10 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>8498715.52</v>
+        <v>8498715.520000001</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>0.0015285099457945</v>
+        <v>0.001533718495646506</v>
       </c>
     </row>
   </sheetData>
@@ -792,25 +792,25 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>660093103.5899988</v>
+        <v>656778058.7399985</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>19715277.43999999</v>
+        <v>19630466.84</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>147900975.67</v>
+        <v>139859811.25</v>
       </c>
       <c r="E2" s="6" t="n">
         <v>58132097.06999999</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>385202405.2100001</v>
+        <v>384508509.7100001</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>345912108.5199999</v>
+        <v>344530938.7999999</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>90729503.34999995</v>
+        <v>90349380.20999996</v>
       </c>
       <c r="I2" s="6" t="n">
         <v>1409656.41</v>
@@ -823,7 +823,7 @@
       <c r="M2" s="6" t="n"/>
       <c r="N2" s="6" t="n"/>
       <c r="O2" s="6" t="n">
-        <v>1710656447.699999</v>
+        <v>1696760239.469999</v>
       </c>
     </row>
     <row r="3">
@@ -833,13 +833,13 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>214109201.7799999</v>
+        <v>213971313.9299999</v>
       </c>
       <c r="C3" s="6" t="n">
         <v>206735200.6899998</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>298850088.86</v>
+        <v>298817549.4999999</v>
       </c>
       <c r="E3" s="6" t="n">
         <v>302333078.9600002</v>
@@ -864,7 +864,7 @@
       <c r="M3" s="6" t="n"/>
       <c r="N3" s="6" t="n"/>
       <c r="O3" s="6" t="n">
-        <v>1184136571.64</v>
+        <v>1183966144.43</v>
       </c>
     </row>
     <row r="4">
@@ -874,7 +874,7 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>707141137.6099992</v>
+        <v>706269202.1799991</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>101550074.49</v>
@@ -889,7 +889,7 @@
         <v>32495046.92999998</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>27010882.07000001</v>
+        <v>27005921.91000001</v>
       </c>
       <c r="H4" s="6" t="n">
         <v>9311150.889999995</v>
@@ -907,7 +907,7 @@
       </c>
       <c r="N4" s="6" t="n"/>
       <c r="O4" s="6" t="n">
-        <v>1158055949.129999</v>
+        <v>1157179053.539999</v>
       </c>
     </row>
     <row r="5">
@@ -920,10 +920,10 @@
         <v>25587289.53</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>475189399.67</v>
+        <v>473741371.14</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>232602429.9299999</v>
+        <v>232502231.1199999</v>
       </c>
       <c r="E5" s="6" t="n">
         <v>129793216.2400001</v>
@@ -950,7 +950,7 @@
         <v>28398.06</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>883032115.7499998</v>
+        <v>881483888.4099998</v>
       </c>
     </row>
     <row r="6">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>105066260.93</v>
+        <v>104059579.93</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>219931923.3200001</v>
@@ -972,10 +972,10 @@
         <v>99415058.01000005</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>20043403.3</v>
+        <v>18807403.3</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>6301333.83</v>
+        <v>6179336.67</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>8882510.540000001</v>
@@ -995,7 +995,7 @@
         <v>659564.1</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>488445360.8000002</v>
+        <v>486080682.6400002</v>
       </c>
     </row>
     <row r="7">
@@ -1100,7 +1100,7 @@
         <v>32163</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>2154211.61</v>
+        <v>2128291.61</v>
       </c>
       <c r="I10" s="6" t="n">
         <v>11930.34</v>
@@ -1111,7 +1111,7 @@
       <c r="M10" s="6" t="n"/>
       <c r="N10" s="6" t="n"/>
       <c r="O10" s="6" t="n">
-        <v>3648995.79</v>
+        <v>3623075.79</v>
       </c>
     </row>
     <row r="11">
@@ -1121,25 +1121,25 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>1711996993.439998</v>
+        <v>1706665444.309998</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>1024530207.67</v>
+        <v>1022997368.54</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>845638881.21</v>
+        <v>837464978.62</v>
       </c>
       <c r="E11" s="6" t="n">
         <v>705080134.7700002</v>
       </c>
       <c r="F11" s="6" t="n">
-        <v>499939221.9100001</v>
+        <v>498009326.4100001</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>413773356.4599999</v>
+        <v>412265229.42</v>
       </c>
       <c r="H11" s="6" t="n">
-        <v>118485767.2099999</v>
+        <v>118079724.07</v>
       </c>
       <c r="I11" s="6" t="n">
         <v>102255069.55</v>
@@ -1160,7 +1160,7 @@
         <v>687962.16</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>5560130991.22</v>
+        <v>5541248634.69</v>
       </c>
     </row>
   </sheetData>
@@ -1216,16 +1216,16 @@
         <v>46235</v>
       </c>
       <c r="B2" s="5" t="n">
-        <v>4060</v>
+        <v>4051</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>1206566780.94</v>
+        <v>1197507442.520001</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>1207949631.42</v>
+        <v>1198890293.000001</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>6643</v>
+        <v>6622</v>
       </c>
     </row>
     <row r="3">
@@ -1233,16 +1233,16 @@
         <v>46266</v>
       </c>
       <c r="B3" s="5" t="n">
-        <v>12652</v>
+        <v>12629</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>4353564210.27999</v>
+        <v>4343741192.169991</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>4360210485.709992</v>
+        <v>4350387467.599994</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>21849</v>
+        <v>21800</v>
       </c>
     </row>
   </sheetData>
@@ -1366,16 +1366,16 @@
         <v>46252</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>23363768.00000001</v>
+        <v>17542512.45</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>83181913.34</v>
+        <v>77360657.79000001</v>
       </c>
     </row>
     <row r="7">
@@ -1389,10 +1389,10 @@
         <v>40755485.55</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>123937398.89</v>
+        <v>118116143.34</v>
       </c>
     </row>
     <row r="8">
@@ -1403,13 +1403,13 @@
         <v>136</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>48980509.10000001</v>
+        <v>48980509.1</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>172917907.99</v>
+        <v>167096652.44</v>
       </c>
     </row>
     <row r="9">
@@ -1423,10 +1423,10 @@
         <v>48985944.67000001</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>221903852.66</v>
+        <v>216082597.11</v>
       </c>
     </row>
     <row r="10">
@@ -1434,16 +1434,16 @@
         <v>46258</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>104538076.59</v>
+        <v>104426271.61</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>1091</v>
+        <v>1089</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>326441929.2500001</v>
+        <v>320508868.72</v>
       </c>
     </row>
     <row r="11">
@@ -1451,16 +1451,16 @@
         <v>46259</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>121956218.7600001</v>
+        <v>120720218.7600001</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>1542</v>
+        <v>1538</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>448398148.0100001</v>
+        <v>441229087.4800001</v>
       </c>
     </row>
     <row r="12">
@@ -1468,16 +1468,16 @@
         <v>46260</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>124663790.5699999</v>
+        <v>124271424.2899999</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>2049</v>
+        <v>2043</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>573061938.58</v>
+        <v>565500511.77</v>
       </c>
     </row>
     <row r="13">
@@ -1491,10 +1491,10 @@
         <v>230218076.0000001</v>
       </c>
       <c r="D13" s="5" t="n">
-        <v>2728</v>
+        <v>2722</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>803280014.5800002</v>
+        <v>795718587.7700001</v>
       </c>
     </row>
     <row r="14">
@@ -1502,16 +1502,16 @@
         <v>46262</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>573</v>
+        <v>570</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>200762482.5200002</v>
+        <v>199264570.9100001</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>3301</v>
+        <v>3292</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>1004042497.1</v>
+        <v>994983158.6800002</v>
       </c>
     </row>
     <row r="15">
@@ -1525,10 +1525,10 @@
         <v>202524283.8399999</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>4060</v>
+        <v>4051</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>1206566780.94</v>
+        <v>1197507442.52</v>
       </c>
     </row>
     <row r="16">
@@ -1542,10 +1542,10 @@
         <v>156860550.9599999</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>4705</v>
+        <v>4696</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>1363427331.9</v>
+        <v>1354367993.48</v>
       </c>
     </row>
     <row r="17">
@@ -1559,10 +1559,10 @@
         <v>132009517.2499999</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>5353</v>
+        <v>5344</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>1495436849.15</v>
+        <v>1486377510.73</v>
       </c>
     </row>
     <row r="18">
@@ -1576,10 +1576,10 @@
         <v>192745214.94</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>6108</v>
+        <v>6099</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>1688182064.09</v>
+        <v>1679122725.67</v>
       </c>
     </row>
     <row r="19">
@@ -1593,10 +1593,10 @@
         <v>159974240.2000001</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>6687</v>
+        <v>6678</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>1848156304.29</v>
+        <v>1839096965.87</v>
       </c>
     </row>
     <row r="20">
@@ -1610,10 +1610,10 @@
         <v>172434042.9600001</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>7276</v>
+        <v>7267</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>2020590347.25</v>
+        <v>2011531008.83</v>
       </c>
     </row>
     <row r="21">
@@ -1621,16 +1621,16 @@
         <v>46274</v>
       </c>
       <c r="B21" s="5" t="n">
-        <v>876</v>
+        <v>873</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>217439301.2500001</v>
+        <v>216867877.5800001</v>
       </c>
       <c r="D21" s="5" t="n">
-        <v>8152</v>
+        <v>8140</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>2238029648.5</v>
+        <v>2228398886.41</v>
       </c>
     </row>
     <row r="22">
@@ -1644,10 +1644,10 @@
         <v>180574228.5700001</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>8841</v>
+        <v>8829</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>2418603877.07</v>
+        <v>2408973114.98</v>
       </c>
     </row>
     <row r="23">
@@ -1661,10 +1661,10 @@
         <v>333979556.3299996</v>
       </c>
       <c r="D23" s="5" t="n">
-        <v>9707</v>
+        <v>9695</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>2752583433.4</v>
+        <v>2742952671.309999</v>
       </c>
     </row>
     <row r="24">
@@ -1672,16 +1672,16 @@
         <v>46279</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>341670123.4199995</v>
+        <v>341549138.6199996</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>10628</v>
+        <v>10615</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>3094253556.819999</v>
+        <v>3084501809.929999</v>
       </c>
     </row>
     <row r="25">
@@ -1689,16 +1689,16 @@
         <v>46280</v>
       </c>
       <c r="B25" s="5" t="n">
-        <v>717</v>
+        <v>713</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>256117200.29</v>
+        <v>255925276.6199999</v>
       </c>
       <c r="D25" s="5" t="n">
-        <v>11345</v>
+        <v>11328</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>3350370757.109999</v>
+        <v>3340427086.549999</v>
       </c>
     </row>
     <row r="26">
@@ -1712,10 +1712,10 @@
         <v>208823984.2600001</v>
       </c>
       <c r="D26" s="5" t="n">
-        <v>11952</v>
+        <v>11935</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>3559194741.369999</v>
+        <v>3549251070.809999</v>
       </c>
     </row>
     <row r="27">
@@ -1723,16 +1723,16 @@
         <v>46282</v>
       </c>
       <c r="B27" s="5" t="n">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>216944390.2799999</v>
+        <v>216602633.0599999</v>
       </c>
       <c r="D27" s="5" t="n">
-        <v>12600</v>
+        <v>12581</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>3776139131.649999</v>
+        <v>3765853703.869999</v>
       </c>
     </row>
     <row r="28">
@@ -1740,16 +1740,16 @@
         <v>46283</v>
       </c>
       <c r="B28" s="5" t="n">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>176814644.08</v>
+        <v>176620907.3799999</v>
       </c>
       <c r="D28" s="5" t="n">
-        <v>13105</v>
+        <v>13084</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>3952953775.729999</v>
+        <v>3942474611.249999</v>
       </c>
     </row>
     <row r="29">
@@ -1763,10 +1763,10 @@
         <v>199621412.1999999</v>
       </c>
       <c r="D29" s="5" t="n">
-        <v>13651</v>
+        <v>13630</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>4152575187.929999</v>
+        <v>4142096023.449999</v>
       </c>
     </row>
     <row r="30">
@@ -1774,16 +1774,16 @@
         <v>46287</v>
       </c>
       <c r="B30" s="5" t="n">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>241769545.0099999</v>
+        <v>241564594.5299999</v>
       </c>
       <c r="D30" s="5" t="n">
-        <v>14142</v>
+        <v>14119</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>4394344732.939999</v>
+        <v>4383660617.979999</v>
       </c>
     </row>
     <row r="31">
@@ -1791,16 +1791,16 @@
         <v>46288</v>
       </c>
       <c r="B31" s="5" t="n">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>170776121.6000003</v>
+        <v>166814064.9600003</v>
       </c>
       <c r="D31" s="5" t="n">
-        <v>14600</v>
+        <v>14575</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>4565120854.539999</v>
+        <v>4550474682.939999</v>
       </c>
     </row>
     <row r="32">
@@ -1814,10 +1814,10 @@
         <v>164555333.73</v>
       </c>
       <c r="D32" s="5" t="n">
-        <v>15011</v>
+        <v>14986</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>4729676188.269999</v>
+        <v>4715030016.669998</v>
       </c>
     </row>
     <row r="33">
@@ -1831,10 +1831,10 @@
         <v>192132004.3899999</v>
       </c>
       <c r="D33" s="5" t="n">
-        <v>15440</v>
+        <v>15415</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>4921808192.659999</v>
+        <v>4907162021.059999</v>
       </c>
     </row>
     <row r="34">
@@ -1842,16 +1842,16 @@
         <v>46293</v>
       </c>
       <c r="B34" s="5" t="n">
-        <v>465</v>
+        <v>462</v>
       </c>
       <c r="C34" s="6" t="n">
-        <v>261215944.1799997</v>
+        <v>259339402.7799997</v>
       </c>
       <c r="D34" s="5" t="n">
-        <v>15905</v>
+        <v>15877</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>5183024136.839998</v>
+        <v>5166501423.839998</v>
       </c>
     </row>
     <row r="35">
@@ -1859,16 +1859,16 @@
         <v>46294</v>
       </c>
       <c r="B35" s="5" t="n">
-        <v>448</v>
+        <v>444</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>205501731.7900001</v>
+        <v>203142088.2600001</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>16353</v>
+        <v>16321</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>5388525868.629998</v>
+        <v>5369643512.099998</v>
       </c>
     </row>
     <row r="36">
@@ -1882,10 +1882,10 @@
         <v>171605122.5899999</v>
       </c>
       <c r="D36" s="5" t="n">
-        <v>16712</v>
+        <v>16680</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>5560130991.219998</v>
+        <v>5541248634.689999</v>
       </c>
     </row>
   </sheetData>
@@ -1899,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H131"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1971,19 +1971,19 @@
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>3725</v>
+        <v>3708</v>
       </c>
       <c r="E2" s="6" t="n">
-        <v>1818328948.480002</v>
+        <v>1804355440.970002</v>
       </c>
       <c r="F2" s="8" t="n">
-        <v>0.3270298759779803</v>
+        <v>0.3256225374321153</v>
       </c>
       <c r="G2" s="6" t="n">
-        <v>1822536206.770002</v>
+        <v>1808562699.260002</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>7962</v>
+        <v>7910</v>
       </c>
     </row>
     <row r="3">
@@ -2009,7 +2009,7 @@
         <v>556263012.7899995</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>0.1000449474424962</v>
+        <v>0.1003858605635586</v>
       </c>
       <c r="G3" s="6" t="n">
         <v>556263012.7899995</v>
@@ -2041,7 +2041,7 @@
         <v>526354516.7300001</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.09466584826169855</v>
+        <v>0.09498843156664212</v>
       </c>
       <c r="G4" s="6" t="n">
         <v>526354516.7300001</v>
@@ -2067,19 +2067,19 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>367028515.4799998</v>
+        <v>366021834.4799998</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.0660107677426259</v>
+        <v>0.06605403558118388</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>367028515.4799998</v>
+        <v>366021834.4799998</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="6">
@@ -2105,7 +2105,7 @@
         <v>135995308.97</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>0.02445901170039881</v>
+        <v>0.02454235821843937</v>
       </c>
       <c r="G6" s="6" t="n">
         <v>135995308.97</v>
@@ -2137,7 +2137,7 @@
         <v>114529920.8800002</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.02059842134310402</v>
+        <v>0.02066861251505771</v>
       </c>
       <c r="G7" s="6" t="n">
         <v>114529920.8800002</v>
@@ -2169,7 +2169,7 @@
         <v>109267038.94</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.01965188214316236</v>
+        <v>0.01971884788853421</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>109267038.94</v>
@@ -2195,19 +2195,19 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>103204676.5899999</v>
+        <v>101430712.78</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.01856155489015823</v>
+        <v>0.01830466731722</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>103204676.5899999</v>
+        <v>101430712.78</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>385</v>
+        <v>379</v>
       </c>
     </row>
     <row r="10">
@@ -2233,7 +2233,7 @@
         <v>98697559.51000002</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0177509414195193</v>
+        <v>0.01781142952007631</v>
       </c>
       <c r="G10" s="6" t="n">
         <v>98697559.51000002</v>
@@ -2259,19 +2259,19 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>97139240.76999998</v>
+        <v>97045702.87999998</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>0.01747067486780303</v>
+        <v>0.01751332764107762</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>97139240.76999998</v>
+        <v>97045702.87999998</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>826</v>
+        <v>825</v>
       </c>
     </row>
     <row r="12">
@@ -2297,7 +2297,7 @@
         <v>96979042.92000005</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>0.01744186298364905</v>
+        <v>0.01750129786865726</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>99307724.88000008</v>
@@ -2329,7 +2329,7 @@
         <v>92265957.86000006</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>0.01659420578502506</v>
+        <v>0.01665075219371776</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>92265957.86000006</v>
@@ -2361,7 +2361,7 @@
         <v>88627966.19</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>0.01593990615148319</v>
+        <v>0.01599422296901828</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>88627966.19</v>
@@ -2393,7 +2393,7 @@
         <v>86672827.36</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>0.01558827076140203</v>
+        <v>0.01564138934632895</v>
       </c>
       <c r="G15" s="6" t="n">
         <v>86672827.36</v>
@@ -2419,19 +2419,19 @@
         </is>
       </c>
       <c r="D16" s="5" t="n">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>86396731.06999996</v>
+        <v>86300603.11999996</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>0.01553861432517129</v>
+        <v>0.01557421599524165</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>86396731.06999996</v>
+        <v>86300603.11999996</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>830</v>
+        <v>829</v>
       </c>
     </row>
     <row r="17">
@@ -2457,7 +2457,7 @@
         <v>73207248.91000001</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>0.013166461190501</v>
+        <v>0.01321132721814702</v>
       </c>
       <c r="G17" s="6" t="n">
         <v>73207248.91000001</v>
@@ -2489,7 +2489,7 @@
         <v>72582167.63000001</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>0.01305403914846871</v>
+        <v>0.01309852208681132</v>
       </c>
       <c r="G18" s="6" t="n">
         <v>72582167.63000001</v>
@@ -2521,7 +2521,7 @@
         <v>70901476.99000002</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>0.01275176378073835</v>
+        <v>0.0127952166856643</v>
       </c>
       <c r="G19" s="6" t="n">
         <v>70901476.99000002</v>
@@ -2553,7 +2553,7 @@
         <v>69557111.86000003</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.01250997718755864</v>
+        <v>0.0125526061805908</v>
       </c>
       <c r="G20" s="6" t="n">
         <v>69557111.86000003</v>
@@ -2579,19 +2579,19 @@
         </is>
       </c>
       <c r="D21" s="5" t="n">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>65713431.15000001</v>
+        <v>65613232.34000001</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>0.01181868399391454</v>
+        <v>0.01184087498424815</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>65713431.15000001</v>
+        <v>65613232.34000001</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="22">
@@ -2617,7 +2617,7 @@
         <v>64694522.00000003</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>0.01163543126990337</v>
+        <v>0.0116750801606323</v>
       </c>
       <c r="G22" s="6" t="n">
         <v>64694522.00000003</v>
@@ -2649,7 +2649,7 @@
         <v>57052310.88000005</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>0.01026096524885679</v>
+        <v>0.01029593050974725</v>
       </c>
       <c r="G23" s="6" t="n">
         <v>57052310.88000005</v>
@@ -2681,7 +2681,7 @@
         <v>56299242.04000001</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>0.01012552440381389</v>
+        <v>0.01016002813653743</v>
       </c>
       <c r="G24" s="6" t="n">
         <v>56299242.04000001</v>
@@ -2713,7 +2713,7 @@
         <v>49291465.83000001</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>0.008865162692720035</v>
+        <v>0.008895371617403986</v>
       </c>
       <c r="G25" s="6" t="n">
         <v>49291465.83000001</v>
@@ -2745,7 +2745,7 @@
         <v>36582479.76</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>0.006579427682147664</v>
+        <v>0.006601847737165573</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>36582479.76</v>
@@ -2777,7 +2777,7 @@
         <v>35568282.98</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>0.006397022486730234</v>
+        <v>0.006418820977880528</v>
       </c>
       <c r="G27" s="6" t="n">
         <v>35568282.98</v>
@@ -2809,7 +2809,7 @@
         <v>34551317.37</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>0.006214119312037785</v>
+        <v>0.006235294542406495</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>35584941.38999999</v>
@@ -2841,7 +2841,7 @@
         <v>32164267.91</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>0.005784803984077097</v>
+        <v>0.005804516279713805</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>32164267.91</v>
@@ -2873,7 +2873,7 @@
         <v>31286474.5</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>0.005626931190902598</v>
+        <v>0.005646105519275313</v>
       </c>
       <c r="G30" s="6" t="n">
         <v>31286474.5</v>
@@ -2905,7 +2905,7 @@
         <v>24603509.66</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>0.004424987414658286</v>
+        <v>0.00444006599992177</v>
       </c>
       <c r="G31" s="6" t="n">
         <v>24603509.66</v>
@@ -2931,19 +2931,19 @@
         </is>
       </c>
       <c r="D32" s="5" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>24174018.57999999</v>
+        <v>24132258.67999999</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>0.004347742637389869</v>
+        <v>0.004355021813842512</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>24174018.57999999</v>
+        <v>24132258.67999999</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33">
@@ -2969,7 +2969,7 @@
         <v>16117759</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>0.002898809223281168</v>
+        <v>0.002908687204378025</v>
       </c>
       <c r="G33" s="6" t="n">
         <v>16117759</v>
@@ -3001,7 +3001,7 @@
         <v>16049360.45</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>0.002886507615619764</v>
+        <v>0.002896343677763499</v>
       </c>
       <c r="G34" s="6" t="n">
         <v>16508922.08</v>
@@ -3033,7 +3033,7 @@
         <v>15218123.01</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>0.002737008001076042</v>
+        <v>0.002746334628395783</v>
       </c>
       <c r="G35" s="6" t="n">
         <v>15218123.01</v>
@@ -3065,7 +3065,7 @@
         <v>14385659.14</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>0.002587287810793736</v>
+        <v>0.002596104251655691</v>
       </c>
       <c r="G36" s="6" t="n">
         <v>14385659.15</v>
@@ -3097,7 +3097,7 @@
         <v>13725820.76</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>0.002468614639056964</v>
+        <v>0.002477026689268543</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>13725820.76</v>
@@ -3129,7 +3129,7 @@
         <v>13372467.61</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>0.002405063411476538</v>
+        <v>0.002413258904551594</v>
       </c>
       <c r="G38" s="6" t="n">
         <v>13372467.61</v>
@@ -3161,7 +3161,7 @@
         <v>11154160.89</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>0.002006096782182565</v>
+        <v>0.002012932756738502</v>
       </c>
       <c r="G39" s="6" t="n">
         <v>11154160.89</v>
@@ -3193,7 +3193,7 @@
         <v>10556313.58</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>0.001898572820796752</v>
+        <v>0.001905042396746841</v>
       </c>
       <c r="G40" s="6" t="n">
         <v>10556313.58</v>
@@ -3225,7 +3225,7 @@
         <v>10011272.7</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>0.001800546195010297</v>
+        <v>0.001806681735471355</v>
       </c>
       <c r="G41" s="6" t="n">
         <v>10011272.7</v>
@@ -3257,7 +3257,7 @@
         <v>9987587.629999999</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>0.001796286390693204</v>
+        <v>0.001802407415446852</v>
       </c>
       <c r="G42" s="6" t="n">
         <v>9987587.629999999</v>
@@ -3289,7 +3289,7 @@
         <v>9377633.550000001</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>0.001686585003987895</v>
+        <v>0.001692332210342087</v>
       </c>
       <c r="G43" s="6" t="n">
         <v>9377633.550000001</v>
@@ -3321,7 +3321,7 @@
         <v>8927355.92</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>0.001605601726667444</v>
+        <v>0.00161107297443971</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>8927355.92</v>
@@ -3353,7 +3353,7 @@
         <v>8847336.98</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>0.001591210170042905</v>
+        <v>0.001596632377152836</v>
       </c>
       <c r="G45" s="6" t="n">
         <v>8847336.98</v>
@@ -3385,7 +3385,7 @@
         <v>8837550.899999999</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>0.001589450125177873</v>
+        <v>0.001594866334759658</v>
       </c>
       <c r="G46" s="6" t="n">
         <v>8837550.899999999</v>
@@ -3417,7 +3417,7 @@
         <v>8557697.060000001</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>0.001539117886523439</v>
+        <v>0.001544362583989836</v>
       </c>
       <c r="G47" s="6" t="n">
         <v>8557697.060000001</v>
@@ -3449,7 +3449,7 @@
         <v>8115794.890000002</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>0.001459640951412053</v>
+        <v>0.001464614823307605</v>
       </c>
       <c r="G48" s="6" t="n">
         <v>8115794.890000002</v>
@@ -3481,7 +3481,7 @@
         <v>7899094.720000001</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>0.001420667018901795</v>
+        <v>0.001425508083241226</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>7899094.720000001</v>
@@ -3513,7 +3513,7 @@
         <v>7733461.810000001</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>0.001390877629000451</v>
+        <v>0.001395617183027313</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>7733461.810000001</v>
@@ -3545,7 +3545,7 @@
         <v>7459531.1</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>0.001341610676399412</v>
+        <v>0.001346182348379196</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>7459531.1</v>
@@ -3557,33 +3557,33 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Sistema Cresol</t>
+          <t>Sistema Sicredi</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Coop. Cresol Rio Grande Do Sul</t>
+          <t>Coop. Sicredi Fronteir Pr/Sc/Sp</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>06139650</t>
+          <t>82527557</t>
         </is>
       </c>
       <c r="D52" s="5" t="n">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E52" s="6" t="n">
-        <v>7221775.340000002</v>
+        <v>6812452.689999999</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>0.001298849856487896</v>
+        <v>0.001229407510674012</v>
       </c>
       <c r="G52" s="6" t="n">
-        <v>7221775.340000002</v>
+        <v>6812452.689999999</v>
       </c>
       <c r="H52" s="5" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="53">
@@ -3594,188 +3594,188 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Coop. Sicredi Fronteir Pr/Sc/Sp</t>
+          <t>Coop. Sicredi Agroempresarial</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>82527557</t>
+          <t>79457883</t>
         </is>
       </c>
       <c r="D53" s="5" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>6812452.689999999</v>
+        <v>6807417.91</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>0.001225232409228765</v>
+        <v>0.001228498910405026</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>6812452.689999999</v>
+        <v>6807417.91</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Sistema Sicredi</t>
+          <t>Sistema Cresol</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Coop. Sicredi Agroempresarial</t>
+          <t>Coop. Cresol Confiança</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>79457883</t>
+          <t>07252614</t>
         </is>
       </c>
       <c r="D54" s="5" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>6807417.91</v>
+        <v>6663937.240000001</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>0.001224326894591079</v>
+        <v>0.001202605708446578</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>6807417.91</v>
+        <v>6663937.240000001</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>12</v>
+        <v>43</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Sistema Cresol</t>
+          <t>Sistema Sicredi</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Coop. Cresol Confiança</t>
+          <t>Coop. Sicredi Biomas</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>07252614</t>
+          <t>33022690</t>
         </is>
       </c>
       <c r="D55" s="5" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>6663937.240000001</v>
+        <v>6549301.34</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>0.001198521626652865</v>
+        <v>0.001181917970437072</v>
       </c>
       <c r="G55" s="6" t="n">
-        <v>6663937.240000001</v>
+        <v>6549301.34</v>
       </c>
       <c r="H55" s="5" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Sistema Sicredi</t>
+          <t>Sistema Sicoob</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Coop. Sicredi Biomas</t>
+          <t>Cc Noroeste De Minas</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>33022690</t>
+          <t>86564051</t>
         </is>
       </c>
       <c r="D56" s="5" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E56" s="6" t="n">
-        <v>6549301.34</v>
+        <v>6439449.65</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>0.001177904144766013</v>
+        <v>0.001162093613646385</v>
       </c>
       <c r="G56" s="6" t="n">
-        <v>6549301.34</v>
+        <v>6439449.65</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Sistema Sicoob</t>
+          <t>Sistema Sicredi</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cc Noroeste De Minas</t>
+          <t>Coop. Sicredi Vale Do Piquiri</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>86564051</t>
+          <t>81099491</t>
         </is>
       </c>
       <c r="D57" s="5" t="n">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>6439449.65</v>
+        <v>6089669.89</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>0.001158147112031809</v>
+        <v>0.001098970699830487</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>6439449.65</v>
+        <v>6089669.89</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>6</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Sistema Sicredi</t>
+          <t>Sistema Cresol</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Coop. Sicredi Vale Do Piquiri</t>
+          <t>Coop. Cresol Rio Grande Do Sul</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>81099491</t>
+          <t>06139650</t>
         </is>
       </c>
       <c r="D58" s="5" t="n">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>6089669.89</v>
+        <v>5985775.34</v>
       </c>
       <c r="F58" s="8" t="n">
-        <v>0.001095238565353261</v>
+        <v>0.00108022139676735</v>
       </c>
       <c r="G58" s="6" t="n">
-        <v>6089669.89</v>
+        <v>5985775.34</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59">
@@ -3801,7 +3801,7 @@
         <v>5868069.67</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>0.001055383349648824</v>
+        <v>0.001058979673509684</v>
       </c>
       <c r="G59" s="6" t="n">
         <v>5868069.67</v>
@@ -3833,7 +3833,7 @@
         <v>5672646.92</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>0.001020236201081894</v>
+        <v>0.001023712757533998</v>
       </c>
       <c r="G60" s="6" t="n">
         <v>5672646.92</v>
@@ -3865,7 +3865,7 @@
         <v>4398993.290000001</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>0.0007911672039645197</v>
+        <v>0.0007938631849978518</v>
       </c>
       <c r="G61" s="6" t="n">
         <v>4398993.290000001</v>
@@ -3897,7 +3897,7 @@
         <v>4195364.439999999</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>0.0007545441729025624</v>
+        <v>0.000757115357310565</v>
       </c>
       <c r="G62" s="6" t="n">
         <v>4195364.439999999</v>
@@ -3929,7 +3929,7 @@
         <v>4060334</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>0.0007302586946983211</v>
+        <v>0.0007327471239209521</v>
       </c>
       <c r="G63" s="6" t="n">
         <v>4060334</v>
@@ -3961,7 +3961,7 @@
         <v>4000000</v>
       </c>
       <c r="F64" s="8" t="n">
-        <v>0.0007194075114986316</v>
+        <v>0.0007218589642339297</v>
       </c>
       <c r="G64" s="6" t="n">
         <v>4000000</v>
@@ -3993,7 +3993,7 @@
         <v>3924328.7</v>
       </c>
       <c r="F65" s="8" t="n">
-        <v>0.0007057978860924149</v>
+        <v>0.0007082029626738709</v>
       </c>
       <c r="G65" s="6" t="n">
         <v>3924328.7</v>
@@ -4025,7 +4025,7 @@
         <v>3870115.25</v>
       </c>
       <c r="F66" s="8" t="n">
-        <v>0.0006960474953038511</v>
+        <v>0.000698419346457734</v>
       </c>
       <c r="G66" s="6" t="n">
         <v>3870115.25</v>
@@ -4057,7 +4057,7 @@
         <v>3622091.02</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>0.000651439871779935</v>
+        <v>0.0006536597180145545</v>
       </c>
       <c r="G67" s="6" t="n">
         <v>3622091.02</v>
@@ -4089,7 +4089,7 @@
         <v>3556321.79</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>0.0006396111522580648</v>
+        <v>0.0006417906909529887</v>
       </c>
       <c r="G68" s="6" t="n">
         <v>3556321.79</v>
@@ -4121,7 +4121,7 @@
         <v>3401844.75</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>0.0006118281665255461</v>
+        <v>0.0006139130319299078</v>
       </c>
       <c r="G69" s="6" t="n">
         <v>3401844.75</v>
@@ -4153,7 +4153,7 @@
         <v>3363060.78</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>0.0006048527966896116</v>
+        <v>0.0006069138928266379</v>
       </c>
       <c r="G70" s="6" t="n">
         <v>3363060.78</v>
@@ -4185,7 +4185,7 @@
         <v>3350406.63</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>0.0006025769240492041</v>
+        <v>0.0006046302649235727</v>
       </c>
       <c r="G71" s="6" t="n">
         <v>3350406.63</v>
@@ -4217,7 +4217,7 @@
         <v>3343181.09</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>0.0006012773971115456</v>
+        <v>0.000603326309718465</v>
       </c>
       <c r="G72" s="6" t="n">
         <v>3343181.09</v>
@@ -4249,7 +4249,7 @@
         <v>3034513.56</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>0.0005457629622021132</v>
+        <v>0.0005476227038438535</v>
       </c>
       <c r="G73" s="6" t="n">
         <v>3034513.56</v>
@@ -4281,7 +4281,7 @@
         <v>2963611.29</v>
       </c>
       <c r="F74" s="8" t="n">
-        <v>0.0005330110557970374</v>
+        <v>0.0005348273440478451</v>
       </c>
       <c r="G74" s="6" t="n">
         <v>2963611.29</v>
@@ -4313,7 +4313,7 @@
         <v>2906644</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>0.0005227653817131071</v>
+        <v>0.0005245467568091916</v>
       </c>
       <c r="G75" s="6" t="n">
         <v>2906644</v>
@@ -4345,7 +4345,7 @@
         <v>2798061.49</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>0.0005032366133852633</v>
+        <v>0.0005049514422585615</v>
       </c>
       <c r="G76" s="6" t="n">
         <v>2798061.49</v>
@@ -4377,7 +4377,7 @@
         <v>2745408.56</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>0.0004937668850491603</v>
+        <v>0.0004954494448801411</v>
       </c>
       <c r="G77" s="6" t="n">
         <v>2745408.56</v>
@@ -4409,7 +4409,7 @@
         <v>2718616.13</v>
       </c>
       <c r="F78" s="8" t="n">
-        <v>0.000488948216200835</v>
+        <v>0.0004906143559378636</v>
       </c>
       <c r="G78" s="6" t="n">
         <v>2718616.13</v>
@@ -4441,7 +4441,7 @@
         <v>2585961.65</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>0.0004650900588643489</v>
+        <v>0.000466674899554416</v>
       </c>
       <c r="G79" s="6" t="n">
         <v>2585961.65</v>
@@ -4467,19 +4467,19 @@
         </is>
       </c>
       <c r="D80" s="5" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>2542117.48</v>
+        <v>2516197.48</v>
       </c>
       <c r="F80" s="8" t="n">
-        <v>0.000457204602555993</v>
+        <v>0.0004540849266802059</v>
       </c>
       <c r="G80" s="6" t="n">
-        <v>2542117.48</v>
+        <v>2516197.48</v>
       </c>
       <c r="H80" s="5" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="81">
@@ -4505,7 +4505,7 @@
         <v>2431698</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>0.0004373454517240498</v>
+        <v>0.0004388357499024296</v>
       </c>
       <c r="G81" s="6" t="n">
         <v>2431698</v>
@@ -4537,7 +4537,7 @@
         <v>2405904.93</v>
       </c>
       <c r="F82" s="8" t="n">
-        <v>0.0004327065196483974</v>
+        <v>0.0004341810102037763</v>
       </c>
       <c r="G82" s="6" t="n">
         <v>2405904.93</v>
@@ -4569,7 +4569,7 @@
         <v>2381834.3</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>0.0004283773716412712</v>
+        <v>0.0004298371101937117</v>
       </c>
       <c r="G83" s="6" t="n">
         <v>2381834.3</v>
@@ -4601,7 +4601,7 @@
         <v>2297143.84</v>
       </c>
       <c r="F84" s="8" t="n">
-        <v>0.0004131456333722026</v>
+        <v>0.0004145534682596879</v>
       </c>
       <c r="G84" s="6" t="n">
         <v>2297143.84</v>
@@ -4633,7 +4633,7 @@
         <v>2280025.15</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>0.0004100668048289485</v>
+        <v>0.0004114641483015775</v>
       </c>
       <c r="G85" s="6" t="n">
         <v>2280025.15</v>
@@ -4665,7 +4665,7 @@
         <v>2246704.31</v>
       </c>
       <c r="F86" s="8" t="n">
-        <v>0.0004040739891825875</v>
+        <v>0.0004054509115391264</v>
       </c>
       <c r="G86" s="6" t="n">
         <v>2246704.31</v>
@@ -4697,7 +4697,7 @@
         <v>2190166.35</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>0.0003939055309053853</v>
+        <v>0.0003952478032277516</v>
       </c>
       <c r="G87" s="6" t="n">
         <v>2190166.35</v>
@@ -4729,7 +4729,7 @@
         <v>2179477.99</v>
       </c>
       <c r="F88" s="8" t="n">
-        <v>0.0003919832092879849</v>
+        <v>0.0003933189311080118</v>
       </c>
       <c r="G88" s="6" t="n">
         <v>2179477.99</v>
@@ -4761,7 +4761,7 @@
         <v>2124475.56</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>0.0003820909189648155</v>
+        <v>0.0003833929318204744</v>
       </c>
       <c r="G89" s="6" t="n">
         <v>2124475.56</v>
@@ -4793,7 +4793,7 @@
         <v>2050145.25</v>
       </c>
       <c r="F90" s="8" t="n">
-        <v>0.00036872247312831</v>
+        <v>0.0003699789316735277</v>
       </c>
       <c r="G90" s="6" t="n">
         <v>2050145.25</v>
@@ -4825,7 +4825,7 @@
         <v>2024934.78</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>0.0003641883227567072</v>
+        <v>0.000365429330733015</v>
       </c>
       <c r="G91" s="6" t="n">
         <v>2024934.78</v>
@@ -4857,7 +4857,7 @@
         <v>1906962.81</v>
       </c>
       <c r="F92" s="8" t="n">
-        <v>0.0003429708424156344</v>
+        <v>0.000344139549714806</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>1906962.81</v>
@@ -4889,7 +4889,7 @@
         <v>1810605.42</v>
       </c>
       <c r="F93" s="8" t="n">
-        <v>0.0003256407848770336</v>
+        <v>0.0003267504382793848</v>
       </c>
       <c r="G93" s="6" t="n">
         <v>1810605.42</v>
@@ -4921,7 +4921,7 @@
         <v>1798306.94</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>0.0003234288801540297</v>
+        <v>0.0003245309962707719</v>
       </c>
       <c r="G94" s="6" t="n">
         <v>1798306.94</v>
@@ -4953,7 +4953,7 @@
         <v>1629638.48</v>
       </c>
       <c r="F95" s="8" t="n">
-        <v>0.0002930935408848031</v>
+        <v>0.0002940922863121388</v>
       </c>
       <c r="G95" s="6" t="n">
         <v>1629638.48</v>
@@ -4965,30 +4965,30 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Sistema Cresol</t>
+          <t>Sistema Sicoob</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Coop. Cresol Ativa</t>
+          <t>Ccla Sul Minas-Sicoob Credivas</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>07946451</t>
+          <t>01604998</t>
         </is>
       </c>
       <c r="D96" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E96" s="6" t="n">
-        <v>1586687.16</v>
+        <v>1466488.63</v>
       </c>
       <c r="F96" s="8" t="n">
-        <v>0.0002853686653256077</v>
+        <v>0.0002646494908781586</v>
       </c>
       <c r="G96" s="6" t="n">
-        <v>1586687.16</v>
+        <v>1466488.63</v>
       </c>
       <c r="H96" s="5" t="n">
         <v>4</v>
@@ -5002,28 +5002,28 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Ccla Sul Minas-Sicoob Credivas</t>
+          <t>Cclaa Itaipu Sicoob Creditaipu</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>01604998</t>
+          <t>81014060</t>
         </is>
       </c>
       <c r="D97" s="5" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E97" s="6" t="n">
-        <v>1466488.63</v>
+        <v>1440241.82</v>
       </c>
       <c r="F97" s="8" t="n">
-        <v>0.0002637507339873343</v>
+        <v>0.0002599128671078975</v>
       </c>
       <c r="G97" s="6" t="n">
-        <v>1466488.63</v>
+        <v>1440241.82</v>
       </c>
       <c r="H97" s="5" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="98">
@@ -5043,51 +5043,51 @@
         </is>
       </c>
       <c r="D98" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E98" s="6" t="n">
-        <v>1452174.75</v>
+        <v>1419635.39</v>
       </c>
       <c r="F98" s="8" t="n">
-        <v>0.0002611763557896618</v>
+        <v>0.0002561941330538077</v>
       </c>
       <c r="G98" s="6" t="n">
-        <v>1452174.75</v>
+        <v>1419635.39</v>
       </c>
       <c r="H98" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Sistema Sicoob</t>
+          <t>Sistema Cresol</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Cclaa Itaipu Sicoob Creditaipu</t>
+          <t>Coop. Cresol Fronteiras Pr/Sc/Sp/Es</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>81014060</t>
+          <t>05276770</t>
         </is>
       </c>
       <c r="D99" s="5" t="n">
         <v>9</v>
       </c>
       <c r="E99" s="6" t="n">
-        <v>1440241.82</v>
+        <v>1344819.58</v>
       </c>
       <c r="F99" s="8" t="n">
-        <v>0.000259030195920615</v>
+        <v>0.0002426925172750771</v>
       </c>
       <c r="G99" s="6" t="n">
-        <v>1440241.82</v>
+        <v>1344819.58</v>
       </c>
       <c r="H99" s="5" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="100">
@@ -5098,28 +5098,28 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Coop. Cresol Fronteiras Pr/Sc/Sp/Es</t>
+          <t>Coop. Cresol Jacutinga</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>05276770</t>
+          <t>02904125</t>
         </is>
       </c>
       <c r="D100" s="5" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E100" s="6" t="n">
-        <v>1344819.58</v>
+        <v>1238405.86</v>
       </c>
       <c r="F100" s="8" t="n">
-        <v>0.0002418683268656087</v>
+        <v>0.0002234885928502072</v>
       </c>
       <c r="G100" s="6" t="n">
-        <v>1344819.58</v>
+        <v>1238405.86</v>
       </c>
       <c r="H100" s="5" t="n">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="101">
@@ -5130,28 +5130,28 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Coop. Cresol Jacutinga</t>
+          <t>Coop. Cresol Ativa</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>02904125</t>
+          <t>07946451</t>
         </is>
       </c>
       <c r="D101" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E101" s="6" t="n">
-        <v>1238405.86</v>
+        <v>1206564.02</v>
       </c>
       <c r="F101" s="8" t="n">
-        <v>0.0002227296194919807</v>
+        <v>0.0002177422634397816</v>
       </c>
       <c r="G101" s="6" t="n">
-        <v>1238405.86</v>
+        <v>1206564.02</v>
       </c>
       <c r="H101" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
@@ -5177,7 +5177,7 @@
         <v>1110448.69</v>
       </c>
       <c r="F102" s="8" t="n">
-        <v>0.0001997162821799539</v>
+        <v>0.000200396835299581</v>
       </c>
       <c r="G102" s="6" t="n">
         <v>1110448.69</v>
@@ -5209,7 +5209,7 @@
         <v>1095224.24</v>
       </c>
       <c r="F103" s="8" t="n">
-        <v>0.000196978136257845</v>
+        <v>0.0001976493588725732</v>
       </c>
       <c r="G103" s="6" t="n">
         <v>1095224.24</v>
@@ -5241,7 +5241,7 @@
         <v>956606</v>
       </c>
       <c r="F104" s="8" t="n">
-        <v>0.000172047385486165</v>
+        <v>0.0001726336540849906</v>
       </c>
       <c r="G104" s="6" t="n">
         <v>956606</v>
@@ -5273,7 +5273,7 @@
         <v>853234</v>
       </c>
       <c r="F105" s="8" t="n">
-        <v>0.0001534557371665059</v>
+        <v>0.0001539786528722932</v>
       </c>
       <c r="G105" s="6" t="n">
         <v>853234</v>
@@ -5305,7 +5305,7 @@
         <v>830126.0700000001</v>
       </c>
       <c r="F106" s="8" t="n">
-        <v>0.0001492997325622097</v>
+        <v>0.0001498084862684456</v>
       </c>
       <c r="G106" s="6" t="n">
         <v>830126.0700000001</v>
@@ -5337,7 +5337,7 @@
         <v>762050</v>
       </c>
       <c r="F107" s="8" t="n">
-        <v>0.000137056123534383</v>
+        <v>0.0001375231559236165</v>
       </c>
       <c r="G107" s="6" t="n">
         <v>762050</v>
@@ -5369,7 +5369,7 @@
         <v>735875.9099999999</v>
       </c>
       <c r="F108" s="8" t="n">
-        <v>0.0001323486642962227</v>
+        <v>0.0001327996555493251</v>
       </c>
       <c r="G108" s="6" t="n">
         <v>735875.9099999999</v>
@@ -5401,7 +5401,7 @@
         <v>627388.27</v>
       </c>
       <c r="F109" s="8" t="n">
-        <v>0.0001128369585160329</v>
+        <v>0.0001132214616886793</v>
       </c>
       <c r="G109" s="6" t="n">
         <v>627388.27</v>
@@ -5433,7 +5433,7 @@
         <v>500000</v>
       </c>
       <c r="F110" s="8" t="n">
-        <v>8.992593893732895e-05</v>
+        <v>9.023237052924121e-05</v>
       </c>
       <c r="G110" s="6" t="n">
         <v>500000</v>
@@ -5465,7 +5465,7 @@
         <v>404770.68</v>
       </c>
       <c r="F111" s="8" t="n">
-        <v>7.279876690660223e-05</v>
+        <v>7.304683595426584e-05</v>
       </c>
       <c r="G111" s="6" t="n">
         <v>404770.68</v>
@@ -5497,7 +5497,7 @@
         <v>376149.05</v>
       </c>
       <c r="F112" s="8" t="n">
-        <v>6.765111300326859e-05</v>
+        <v>6.788164090764416e-05</v>
       </c>
       <c r="G112" s="6" t="n">
         <v>376149.05</v>
@@ -5529,7 +5529,7 @@
         <v>366472.33</v>
       </c>
       <c r="F113" s="8" t="n">
-        <v>6.591073673960133e-05</v>
+        <v>6.613533413854871e-05</v>
       </c>
       <c r="G113" s="6" t="n">
         <v>366472.33</v>
@@ -5561,7 +5561,7 @@
         <v>356062.78</v>
       </c>
       <c r="F114" s="8" t="n">
-        <v>6.403855962427118e-05</v>
+        <v>6.42567773932634e-05</v>
       </c>
       <c r="G114" s="6" t="n">
         <v>356062.78</v>
@@ -5590,13 +5590,13 @@
         <v>6</v>
       </c>
       <c r="E115" s="6" t="n">
-        <v>347843.57</v>
+        <v>347843.5699999999</v>
       </c>
       <c r="F115" s="8" t="n">
-        <v>6.256031927112501e-05</v>
+        <v>6.27734997889081e-05</v>
       </c>
       <c r="G115" s="6" t="n">
-        <v>347843.57</v>
+        <v>347843.5699999999</v>
       </c>
       <c r="H115" s="5" t="n">
         <v>7</v>
@@ -5625,7 +5625,7 @@
         <v>345277.73</v>
       </c>
       <c r="F116" s="8" t="n">
-        <v>6.20988481287991e-05</v>
+        <v>6.23104561377106e-05</v>
       </c>
       <c r="G116" s="6" t="n">
         <v>345277.73</v>
@@ -5657,7 +5657,7 @@
         <v>344207.72</v>
       </c>
       <c r="F117" s="8" t="n">
-        <v>6.190640482095443e-05</v>
+        <v>6.211735706013061e-05</v>
       </c>
       <c r="G117" s="6" t="n">
         <v>344207.72</v>
@@ -5689,7 +5689,7 @@
         <v>311153.02</v>
       </c>
       <c r="F118" s="8" t="n">
-        <v>5.596145495337099e-05</v>
+        <v>5.615214918386481e-05</v>
       </c>
       <c r="G118" s="6" t="n">
         <v>311153.02</v>
@@ -5721,7 +5721,7 @@
         <v>296464.94</v>
       </c>
       <c r="F119" s="8" t="n">
-        <v>5.331977618299778e-05</v>
+        <v>5.350146863001853e-05</v>
       </c>
       <c r="G119" s="6" t="n">
         <v>296464.94</v>
@@ -5753,7 +5753,7 @@
         <v>255566.66</v>
       </c>
       <c r="F120" s="8" t="n">
-        <v>4.596414372315422e-05</v>
+        <v>4.612077112008122e-05</v>
       </c>
       <c r="G120" s="6" t="n">
         <v>255566.66</v>
@@ -5785,7 +5785,7 @@
         <v>238958.61</v>
       </c>
       <c r="F121" s="8" t="n">
-        <v>4.2977154742818e-05</v>
+        <v>4.312360367734489e-05</v>
       </c>
       <c r="G121" s="6" t="n">
         <v>238958.61</v>
@@ -5817,7 +5817,7 @@
         <v>146956.65</v>
       </c>
       <c r="F122" s="8" t="n">
-        <v>2.643042946866884e-05</v>
+        <v>2.652049378907203e-05</v>
       </c>
       <c r="G122" s="6" t="n">
         <v>146956.65</v>
@@ -5849,7 +5849,7 @@
         <v>138480.34</v>
       </c>
       <c r="F123" s="8" t="n">
-        <v>2.49059491977211e-05</v>
+        <v>2.499081869979061e-05</v>
       </c>
       <c r="G123" s="6" t="n">
         <v>138480.34</v>
@@ -5881,7 +5881,7 @@
         <v>134840.12</v>
       </c>
       <c r="F124" s="8" t="n">
-        <v>2.425124879484422e-05</v>
+        <v>2.433388734009469e-05</v>
       </c>
       <c r="G124" s="6" t="n">
         <v>134840.12</v>
@@ -5913,7 +5913,7 @@
         <v>131555.61</v>
       </c>
       <c r="F125" s="8" t="n">
-        <v>2.366052350344612e-05</v>
+        <v>2.37411490934407e-05</v>
       </c>
       <c r="G125" s="6" t="n">
         <v>131555.61</v>
@@ -5930,25 +5930,25 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Cc União Centro Oeste Ltda</t>
+          <t>Coop. Novos Campos</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>26178111</t>
+          <t>78862083</t>
         </is>
       </c>
       <c r="D126" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E126" s="6" t="n">
-        <v>121997.16</v>
+        <v>83442.06</v>
       </c>
       <c r="F126" s="8" t="n">
-        <v>2.19414183213751e-05</v>
+        <v>1.505834975128635e-05</v>
       </c>
       <c r="G126" s="6" t="n">
-        <v>121997.16</v>
+        <v>83442.06</v>
       </c>
       <c r="H126" s="5" t="n">
         <v>1</v>
@@ -5962,25 +5962,25 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Coop. Novos Campos</t>
+          <t>Coop. Sicoob Credicapital</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>78862083</t>
+          <t>04529074</t>
         </is>
       </c>
       <c r="D127" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E127" s="6" t="n">
-        <v>83442.06</v>
+        <v>70328.85000000001</v>
       </c>
       <c r="F127" s="8" t="n">
-        <v>1.500721118472988e-05</v>
+        <v>1.269187770419085e-05</v>
       </c>
       <c r="G127" s="6" t="n">
-        <v>83442.06</v>
+        <v>70328.85000000001</v>
       </c>
       <c r="H127" s="5" t="n">
         <v>1</v>
@@ -5994,60 +5994,60 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Coop. Sicoob Credicapital</t>
+          <t>Ccla Sicoob Valcredi Sul</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>04529074</t>
+          <t>02090126</t>
         </is>
       </c>
       <c r="D128" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E128" s="6" t="n">
-        <v>70328.85000000001</v>
+        <v>39576.28</v>
       </c>
       <c r="F128" s="8" t="n">
-        <v>1.264877574126513e-05</v>
+        <v>7.142123122257996e-06</v>
       </c>
       <c r="G128" s="6" t="n">
-        <v>70328.85000000001</v>
+        <v>39576.28</v>
       </c>
       <c r="H128" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Sistema Sicoob</t>
+          <t>Sistema Sicredi</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Ccla Sicoob Valcredi Sul</t>
+          <t>Coop. Sicredi Integração Pr/Sc</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>02090126</t>
+          <t>81054686</t>
         </is>
       </c>
       <c r="D129" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E129" s="6" t="n">
-        <v>39576.28</v>
+        <v>38825.59</v>
       </c>
       <c r="F129" s="8" t="n">
-        <v>7.117868277293265e-06</v>
+        <v>7.006650045792803e-06</v>
       </c>
       <c r="G129" s="6" t="n">
-        <v>39576.28</v>
+        <v>38825.59</v>
       </c>
       <c r="H129" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
@@ -6058,59 +6058,27 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Coop. Sicredi Integração Pr/Sc</t>
+          <t>Coop. Sicredi Vlr Sustent Pr/Sp</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>81054686</t>
+          <t>81706616</t>
         </is>
       </c>
       <c r="D130" s="5" t="n">
         <v>1</v>
       </c>
       <c r="E130" s="6" t="n">
-        <v>38825.59</v>
+        <v>3995.54</v>
       </c>
       <c r="F130" s="8" t="n">
-        <v>6.982855271091538e-06</v>
+        <v>7.210540914888088e-07</v>
       </c>
       <c r="G130" s="6" t="n">
-        <v>38825.59</v>
+        <v>3995.54</v>
       </c>
       <c r="H130" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Sistema Sicredi</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Coop. Sicredi Vlr Sustent Pr/Sp</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>81706616</t>
-        </is>
-      </c>
-      <c r="D131" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="E131" s="6" t="n">
-        <v>3995.54</v>
-      </c>
-      <c r="F131" s="8" t="n">
-        <v>7.186053721233105e-07</v>
-      </c>
-      <c r="G131" s="6" t="n">
-        <v>3995.54</v>
-      </c>
-      <c r="H131" s="5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6192,22 +6160,22 @@
         </is>
       </c>
       <c r="C2" s="5" t="n">
-        <v>15041</v>
+        <v>15016</v>
       </c>
       <c r="D2" s="6" t="n">
-        <v>4590230446.189997</v>
+        <v>4574542409.329998</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>0.8255615656246996</v>
+        <v>0.8255436113607844</v>
       </c>
       <c r="F2" s="6" t="n">
-        <v>4594441959.759997</v>
+        <v>4578753922.9</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>26079</v>
+        <v>26017</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>305181.2011295789</v>
+        <v>304644.5397795683</v>
       </c>
     </row>
     <row r="3">
@@ -6222,22 +6190,22 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>179414476.5899998</v>
+        <v>179381937.2299998</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>0.03226803053261031</v>
+        <v>0.03237211485278086</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>179414476.5899998</v>
+        <v>179381937.2299998</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="H3" s="6" t="n">
-        <v>376130.9781761002</v>
+        <v>376852.8093067223</v>
       </c>
     </row>
     <row r="4">
@@ -6252,22 +6220,22 @@
         </is>
       </c>
       <c r="C4" s="5" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>161294045.09</v>
+        <v>161172047.93</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0.02900903689943624</v>
+        <v>0.02908587189555277</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>162412949.83</v>
+        <v>162290952.67</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>943240.0297660819</v>
+        <v>948070.8701764706</v>
       </c>
     </row>
     <row r="5">
@@ -6282,22 +6250,22 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>121500398</v>
+        <v>120915324.38</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0.02185207474281833</v>
+        <v>0.02182095270423911</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>121500398</v>
+        <v>120915324.38</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>633</v>
+        <v>629</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>230114.3901515152</v>
+        <v>230314.9035809524</v>
       </c>
     </row>
     <row r="6">
@@ -6318,7 +6286,7 @@
         <v>86717466.93000002</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>0.01559629927189405</v>
+        <v>0.01564944521476997</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>86899210.82000002</v>
@@ -6348,7 +6316,7 @@
         <v>81177353.08000001</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>0.01459989939233215</v>
+        <v>0.0146496500033952</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>81198275.19000001</v>
@@ -6372,22 +6340,22 @@
         </is>
       </c>
       <c r="C8" s="5" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>79110033.51000001</v>
+        <v>78103352.50999999</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>0.01422808808550061</v>
+        <v>0.01409490128651652</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>79265684.33</v>
+        <v>78259003.33</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>1551177.127647059</v>
+        <v>1562067.0502</v>
       </c>
     </row>
     <row r="9">
@@ -6402,22 +6370,22 @@
         </is>
       </c>
       <c r="C9" s="5" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>57417120.19</v>
+        <v>55969091.66</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>0.01032657688832643</v>
+        <v>0.01010044763370037</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>57344420.42</v>
+        <v>55896391.89</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>1510976.847105263</v>
+        <v>1512678.152972973</v>
       </c>
     </row>
     <row r="10">
@@ -6438,7 +6406,7 @@
         <v>55050618.36999999</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>0.009900957092005636</v>
+        <v>0.009934695589251384</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>55238366.55999999</v>
@@ -6468,7 +6436,7 @@
         <v>28739195.48</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>0.00516879827568488</v>
+        <v>0.005186411470527308</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>28744945.7</v>
@@ -6498,7 +6466,7 @@
         <v>26973508.82</v>
       </c>
       <c r="E12" s="8" t="n">
-        <v>0.004851236214145647</v>
+        <v>0.004867767284639992</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>26973508.82</v>
@@ -6528,7 +6496,7 @@
         <v>24902365.61</v>
       </c>
       <c r="E13" s="8" t="n">
-        <v>0.004478737218479799</v>
+        <v>0.004493998961552306</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>24988089.22</v>
@@ -6558,7 +6526,7 @@
         <v>15106762.5</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>0.002716979604231462</v>
+        <v>0.002726237982794493</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>15979264.51</v>
@@ -6588,7 +6556,7 @@
         <v>14060726.14</v>
       </c>
       <c r="E15" s="8" t="n">
-        <v>0.00252884800056029</v>
+        <v>0.002537465301949335</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>14060726.14</v>
@@ -6618,7 +6586,7 @@
         <v>7130083.57</v>
       </c>
       <c r="E16" s="8" t="n">
-        <v>0.001282358919467745</v>
+        <v>0.00128672868518539</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>7130083.57</v>
@@ -6648,7 +6616,7 @@
         <v>6344755.919999998</v>
       </c>
       <c r="E17" s="8" t="n">
-        <v>0.001141116266868352</v>
+        <v>0.001145004734182073</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>7569376.159999998</v>
@@ -6678,7 +6646,7 @@
         <v>5572852.069999999</v>
       </c>
       <c r="E18" s="8" t="n">
-        <v>0.001002287909907174</v>
+        <v>0.001005703305769778</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>5511108.939999999</v>
@@ -6708,7 +6676,7 @@
         <v>4369593.489999999</v>
       </c>
       <c r="E19" s="8" t="n">
-        <v>0.00078587959472538</v>
+        <v>0.0007885575577036804</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>4465384.649999999</v>
@@ -6738,7 +6706,7 @@
         <v>4111535.07</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>0.0007394673032870131</v>
+        <v>0.0007419871117604194</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>4111535.07</v>
@@ -6768,7 +6736,7 @@
         <v>2746200.139999999</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>0.0004939092521986482</v>
+        <v>0.000495592297159868</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>2746200.139999999</v>
@@ -6798,7 +6766,7 @@
         <v>2518876.02</v>
       </c>
       <c r="E22" s="8" t="n">
-        <v>0.0004530245823304443</v>
+        <v>0.0004545683087077208</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>2518876.02</v>
@@ -6828,7 +6796,7 @@
         <v>1726457.99</v>
       </c>
       <c r="E23" s="8" t="n">
-        <v>0.0003105067115732074</v>
+        <v>0.000311564794113698</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>1729156.24</v>
@@ -6858,7 +6826,7 @@
         <v>1584685.74</v>
       </c>
       <c r="E24" s="8" t="n">
-        <v>0.0002850087061801919</v>
+        <v>0.0002859799017281696</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>1584685.74</v>
@@ -6888,7 +6856,7 @@
         <v>1294632.41</v>
       </c>
       <c r="E25" s="8" t="n">
-        <v>0.000232842070095894</v>
+        <v>0.000233635502636569</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>1294632.41</v>
@@ -6918,7 +6886,7 @@
         <v>1036802.3</v>
       </c>
       <c r="E26" s="8" t="n">
-        <v>0.0001864708406397644</v>
+        <v>0.000187106258598339</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>1036802.3</v>
@@ -7263,7 +7231,7 @@
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>6326534.03</v>
+        <v>4878505.5</v>
       </c>
     </row>
     <row r="22">
@@ -7353,7 +7321,7 @@
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>47827648.35999999</v>
+        <v>47705651.2</v>
       </c>
     </row>
     <row r="28">
@@ -7758,7 +7726,7 @@
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>130390630.95</v>
+        <v>130358091.59</v>
       </c>
     </row>
     <row r="55">
@@ -7998,7 +7966,7 @@
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>2621843885.719994</v>
+        <v>2621391276.369994</v>
       </c>
     </row>
     <row r="71">
@@ -8013,7 +7981,7 @@
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>1817750946.100002</v>
+        <v>1803777438.590002</v>
       </c>
     </row>
     <row r="72">
@@ -8043,7 +8011,7 @@
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>64943411.37000001</v>
+        <v>63681491.37000002</v>
       </c>
     </row>
     <row r="74">
@@ -8103,7 +8071,7 @@
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>77949647.5</v>
+        <v>77744697.02</v>
       </c>
     </row>
     <row r="78">
@@ -8118,7 +8086,7 @@
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>19787962.14999999</v>
+        <v>19407839.01</v>
       </c>
     </row>
     <row r="79">
@@ -8208,7 +8176,7 @@
         </is>
       </c>
       <c r="C84" s="6" t="n">
-        <v>64168523.72</v>
+        <v>63161842.72</v>
       </c>
     </row>
     <row r="85">
@@ -8589,7 +8557,7 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>56305524.67999999</v>
+        <v>54857496.14999999</v>
       </c>
     </row>
     <row r="17">
@@ -8649,7 +8617,7 @@
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>1530636.38</v>
+        <v>1408639.22</v>
       </c>
     </row>
     <row r="21">
@@ -8844,7 +8812,7 @@
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>4786115.16</v>
+        <v>4808115.16</v>
       </c>
     </row>
     <row r="34">
@@ -8859,7 +8827,7 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>1274153.02</v>
+        <v>1252153.02</v>
       </c>
     </row>
     <row r="35">
@@ -8934,7 +8902,7 @@
         </is>
       </c>
       <c r="C39" s="6" t="n">
-        <v>11527011.61</v>
+        <v>11494472.25</v>
       </c>
     </row>
     <row r="40">
@@ -9069,7 +9037,7 @@
         </is>
       </c>
       <c r="C48" s="6" t="n">
-        <v>6703170.840000001</v>
+        <v>6703170.84</v>
       </c>
     </row>
     <row r="49">
@@ -9099,7 +9067,7 @@
         </is>
       </c>
       <c r="C50" s="6" t="n">
-        <v>1382978103.010001</v>
+        <v>1372680054.960002</v>
       </c>
     </row>
     <row r="51">
@@ -9114,7 +9082,7 @@
         </is>
       </c>
       <c r="C51" s="6" t="n">
-        <v>807846240.3099974</v>
+        <v>807129945.2399973</v>
       </c>
     </row>
     <row r="52">
@@ -9129,7 +9097,7 @@
         </is>
       </c>
       <c r="C52" s="6" t="n">
-        <v>2399406102.87</v>
+        <v>2394732409.129999</v>
       </c>
     </row>
     <row r="53">
@@ -9159,7 +9127,7 @@
         </is>
       </c>
       <c r="C54" s="6" t="n">
-        <v>21151940.81999999</v>
+        <v>20946990.33999999</v>
       </c>
     </row>
     <row r="55">
@@ -9174,7 +9142,7 @@
         </is>
       </c>
       <c r="C55" s="6" t="n">
-        <v>70198534.29999997</v>
+        <v>69818411.15999997</v>
       </c>
     </row>
     <row r="56">
@@ -9219,7 +9187,7 @@
         </is>
       </c>
       <c r="C58" s="6" t="n">
-        <v>74756144.70999999</v>
+        <v>73749463.70999999</v>
       </c>
     </row>
     <row r="59">
@@ -9630,7 +9598,7 @@
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>6193662.66</v>
+        <v>4745634.13</v>
       </c>
     </row>
     <row r="23">
@@ -9660,7 +9628,7 @@
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>4906644.359999999</v>
+        <v>4906644.359999998</v>
       </c>
     </row>
     <row r="25">
@@ -9675,7 +9643,7 @@
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>87676639.29000002</v>
+        <v>87554642.13000003</v>
       </c>
     </row>
     <row r="26">
@@ -10095,7 +10063,7 @@
         </is>
       </c>
       <c r="C53" s="6" t="n">
-        <v>38826867.48000003</v>
+        <v>38794328.12000003</v>
       </c>
     </row>
     <row r="54">
@@ -10305,7 +10273,7 @@
         </is>
       </c>
       <c r="C67" s="6" t="n">
-        <v>98252015.99000004</v>
+        <v>97016015.99000001</v>
       </c>
     </row>
     <row r="68">
@@ -10335,7 +10303,7 @@
         </is>
       </c>
       <c r="C69" s="6" t="n">
-        <v>1079812611.760002</v>
+        <v>1079674723.910002</v>
       </c>
     </row>
     <row r="70">
@@ -10350,7 +10318,7 @@
         </is>
       </c>
       <c r="C70" s="6" t="n">
-        <v>727562347.9400001</v>
+        <v>727462149.13</v>
       </c>
     </row>
     <row r="71">
@@ -10365,7 +10333,7 @@
         </is>
       </c>
       <c r="C71" s="6" t="n">
-        <v>2310932.09</v>
+        <v>2285012.09</v>
       </c>
     </row>
     <row r="72">
@@ -10380,7 +10348,7 @@
         </is>
       </c>
       <c r="C72" s="6" t="n">
-        <v>1688823384.809999</v>
+        <v>1675307299.72</v>
       </c>
     </row>
     <row r="73">
@@ -10395,7 +10363,7 @@
         </is>
       </c>
       <c r="C73" s="6" t="n">
-        <v>991485620.5699993</v>
+        <v>990813675.4599993</v>
       </c>
     </row>
     <row r="74">
@@ -10455,7 +10423,7 @@
         </is>
       </c>
       <c r="C77" s="6" t="n">
-        <v>13085750.62</v>
+        <v>12705627.48</v>
       </c>
     </row>
     <row r="78">
@@ -10470,7 +10438,7 @@
         </is>
       </c>
       <c r="C78" s="6" t="n">
-        <v>38111006.28999999</v>
+        <v>37906055.80999999</v>
       </c>
     </row>
     <row r="79">
@@ -10500,7 +10468,7 @@
         </is>
       </c>
       <c r="C80" s="6" t="n">
-        <v>67357331.95999999</v>
+        <v>66350650.95999999</v>
       </c>
     </row>
     <row r="81">
@@ -10677,10 +10645,10 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>1863398843.390002</v>
+        <v>1851149670.050002</v>
       </c>
       <c r="D2" s="8" t="n">
-        <v>0.3351357812131575</v>
+        <v>0.3340672458660688</v>
       </c>
     </row>
     <row r="3">
@@ -10695,10 +10663,10 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>1727982781.860005</v>
+        <v>1724040008.190006</v>
       </c>
       <c r="D3" s="8" t="n">
-        <v>0.3107809482525973</v>
+        <v>0.3111284336524733</v>
       </c>
     </row>
     <row r="4">
@@ -10713,10 +10681,10 @@
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>869662533.3899996</v>
+        <v>868870144.1599996</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>0.1564104397474238</v>
+        <v>0.1568004255792806</v>
       </c>
     </row>
     <row r="5">
@@ -10731,10 +10699,10 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>646237347.3299981</v>
+        <v>645216104.6199982</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>0.1162270004700377</v>
+        <v>0.1164387572470107</v>
       </c>
     </row>
     <row r="6">
@@ -10749,10 +10717,10 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>169296946.97</v>
+        <v>169116053.75</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0.03044837383100087</v>
+        <v>0.03051948484882614</v>
       </c>
     </row>
     <row r="7">
@@ -10767,10 +10735,10 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>154429941.3200001</v>
+        <v>154397401.96</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0.02777451494647524</v>
+        <v>0.02786328716481383</v>
       </c>
     </row>
     <row r="8">
@@ -10785,10 +10753,10 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>62066469.43000003</v>
+        <v>61725815.45000003</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0.01116277108003555</v>
+        <v>0.01113933330180793</v>
       </c>
     </row>
     <row r="9">
@@ -10806,7 +10774,7 @@
         <v>48122091.48000001</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0.008654848519934076</v>
+        <v>0.008684340778130805</v>
       </c>
     </row>
     <row r="10">
@@ -10821,10 +10789,10 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>10435320.49</v>
+        <v>10112629.47</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0.001876811986350395</v>
+        <v>0.001824973058723928</v>
       </c>
     </row>
     <row r="11">
@@ -10839,10 +10807,10 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>4233108.110000001</v>
+        <v>4233108.11</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0.0007613324428299441</v>
+        <v>0.000763926758943712</v>
       </c>
     </row>
     <row r="12">
@@ -10860,7 +10828,7 @@
         <v>3089399.09</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0.0005556342278407592</v>
+        <v>0.0005575276068031611</v>
       </c>
     </row>
     <row r="13">
@@ -10878,7 +10846,7 @@
         <v>1176208.32</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>0.0002115432751237966</v>
+        <v>0.0002122641298996327</v>
       </c>
     </row>
   </sheetData>
@@ -11162,13 +11130,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6484F4C4-D5ED-46BB-B6CB-EF82CC799E21}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{66590FB6-5992-4E68-B37E-05037ADB5910}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86F7BC9C-75C8-481F-8CC2-85549B785F32}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C9447050-CC4D-4031-A0A4-6FD97C49750E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2525F93-5B62-4764-9F8F-EA288051146A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{54C0F2BF-4818-4B91-8337-0FFEA37E1B0C}"/>
 </file>
</xml_diff>